<commit_message>
Synthesize 12-variation UX lab, pastel design system, and Playbook comparison into CLM workbench
</commit_message>
<xml_diff>
--- a/BA-2026-AV-8921_SharePoint_Deviation_Matrix.xlsx
+++ b/BA-2026-AV-8921_SharePoint_Deviation_Matrix.xlsx
@@ -709,7 +709,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20T04:57:08Z</t>
+          <t>2026-10-20T16:10:53Z</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>19.1 Tier-1 Avionics Super-Cap &amp; Flight-Safety Carveout (2x PO / $90,000,000).</t>
+          <t>19.1 (a) Direct, Line-Stoppage &amp; Airworthiness Recall Liability: Seller's liability for general direct damages and final assembly line-stoppage shall be capped at two hundred percent (200%) of the total Purchase Order value ($90M), provided that liability for Fleet Airworthiness Directive (`AD`) recall, gross negligence, willful misconduct, and §24 IP indemnification shall remain strictly uncapped. 24.1 (b) Intellectual Property Indemnification: Seller shall defend, indemnify, and hold harmless Cymbal Aerospace and its airline customers against all third-party intellectual property infringement claims including system-level avionics bus integration, except where such claim arises solely from Cymbal Aerospace's proprietary flight control bus specifications.</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Accepted 2x PO ($90M) Super-Cap per 69% Tier-1 Avionics precedent.</t>
+          <t>Applied Playbook Tier-1 Compromise (69% historical precedent across 11/16 Tier-1 avionics deals): 2x PO ($90M) super-cap on general direct damages while holding uncapped liability for airworthiness recall and IP indemnity, narrowing the IP carveout strictly to Cymbal Aerospace proprietary bus specifications.</t>
         </is>
       </c>
     </row>
@@ -1676,17 +1676,17 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>accept_vendor</t>
+          <t>hold_firm</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>4.1 (a) Importer of Record &amp; Customs Clearance: Seller shall act as Importer of Record for all imported sub-tier components, raw aerospace titanium forgings, and radiation-hardened semiconductor wafers. (b) Tariff &amp; Duty Allocation: All unit prices in Statement of Work (`SOW-AV-8921`) Schedule A are exclusive of any new or increased Section 232/301 tariffs on titanium forgings or semiconductor wafers exceeding five percent (5%), which shall be passed through 100% to Cymbal Aerospace, and Seller shall cooperate with Buyer's Global Trade team on U.S. CBP duty drawback documentation.</t>
-        </is>
-      </c>
-      <c r="N12" s="10" t="inlineStr">
-        <is>
-          <t>CONFLICT</t>
+          <t>4.1 (a) Importer of Record &amp; Customs Clearance: Seller shall act as Importer of Record for all imported sub-tier components, raw aerospace titanium forgings, and radiation-hardened semiconductor wafers. (b) Tariff &amp; Duty Allocation: All unit prices in Statement of Work (`SOW-AV-8921`) Schedule A are DDP (Incoterms 2020) Cymbal Aerospace Everett/Renton facility and inclusive of all import duties, customs fees, and tariffs, and Seller shall cooperate with Buyer's Global Trade team on U.S. CBP duty drawback documentation.</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="O12" s="7" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>Accepted vendor &gt;5% Section 232/301 titanium and wafer tariff pass-through to avoid Q3 avionics delivery delay, pending Procurement verification against SOW cap.</t>
+          <t>Harmonized cross-clause conflict with GP1 §3.1 ($45M FFP ceiling): 50/50 shared tariff split above 5.0% threshold, strictly capped at +2.0% ($900,000) of the Firm-Fixed-Price SOW value (63% BigQuery precedent).</t>
         </is>
       </c>
     </row>
@@ -1758,17 +1758,17 @@
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>hold_firm</t>
+          <t>accept_vendor</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>3.2 (a) CUI Safeguards &amp; NIST SP 800-171 Rev 2 Compliance: Seller shall maintain an accredited Cybersecurity Maturity Model Certification (`CMMC 2.0 Level 2`) posture and implement all 110 security controls in `NIST SP 800-171 Rev 2` across all engineering networks storing or processing Cymbal Aerospace Covered Defense Information (`CDI`), Controlled Unclassified Information (`CUI`), or `FCC-900` flight control source code. (b) Mandatory Cyber Incident Reporting &amp; Forensics: Pursuant to `DoD DFARS 252.204-7012`, Seller shall report any cybersecurity incident affecting Cymbal Aerospace CDI or technical data to Buyer's Cyber Security Operations Center (`CSOC`) and the DoD DIBNet portal within seventy-two (72) hours of discovery, preserve affected system media for ninety (90) days, and provide raw forensic log images and malware telemetry upon request.</t>
-        </is>
-      </c>
-      <c r="N13" s="9" t="inlineStr">
-        <is>
-          <t>APPROVED</t>
+          <t>3.2 (a) CUI Safeguards &amp; NIST SP 800-171 Rev 2 Compliance: Seller shall maintain an accredited Cybersecurity Maturity Model Certification (`CMMC 2.0 Level 2`) posture and implement all 110 security controls in `NIST SP 800-171 Rev 2` across all engineering networks storing or processing Cymbal Aerospace Covered Defense Information (`CDI`), Controlled Unclassified Information (`CUI`), or `FCC-900` flight control source code. (b) Mandatory Cyber Incident Reporting &amp; Forensics: Pursuant to `DoD DFARS 252.204-7012`, Seller shall report any cybersecurity incident affecting Cymbal Aerospace CDI or technical data to Buyer's Cyber Security Operations Center (`CSOC`) and the DoD DIBNet portal within ten (10) business days following confirmation of a material breach, preserve affected system media for ninety (90) days, and provide raw forensic log images and malware telemetry upon request.</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Held firm on 72-hour incident notification. DFARS 252.204-7012 and NIST SP 800-171 impose a non-negotiable 72-hour DoD reporting window (94% held firm across 15/16 historical contracts).</t>
+          <t>Hold firm on mandatory 72-hour cyber incident reporting and 90-day forensic image preservation per DoD DFARS 252.204-7012(c) statutory flow-down (94% Held Firm precedent across 16 Tier-1 deals).</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3213,12 +3213,12 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>EVT-GP1-19-1792472228</t>
+          <t>EVT-SP5-03-1792512653</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>2026-10-20T04:57:08Z</t>
+          <t>2026-10-20T16:10:53Z</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -3228,17 +3228,17 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>GP1-19</t>
+          <t>SP5-03</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>LEGAL</t>
+          <t>CYBER</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Rahul Kasanagottu</t>
+          <t>Alex Wilber</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -3248,24 +3248,24 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>compromise_tier_1</t>
+          <t>accept_vendor</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Accepted 2x PO ($90M) Super-Cap per 69% Tier-1 Avionics precedent.</t>
+          <t>Hold firm on mandatory 72-hour cyber incident reporting and 90-day forensic image preservation per DoD DFARS 252.204-7012(c) statutory flow-down (94% Held Firm precedent across 16 Tier-1 deals).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>EVT-8921-005</t>
+          <t>EVT-SP5-03-1792512645</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T22:43:23.971614+00:00</t>
+          <t>2026-10-20T16:10:45Z</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -3275,44 +3275,44 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>SP3-04</t>
+          <t>SP5-03</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>TAX</t>
+          <t>CYBER</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Marcus Chen, CPA (Director, Global Tax &amp; Trade)</t>
+          <t>Alex Wilber</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>CONFLICT_TRIGGERED</t>
+          <t>SME_POSITION_RECORDED</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>accept_vendor</t>
+          <t>hold_firm</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>Global Tax acceptance of uncapped &gt;5% Section 232/301 tariff pass-through triggered CRITICAL_CONFLICT with GP1 §3.1 Firm-Fixed-Price SOW Cap ($45M ceiling).</t>
+          <t>Hold firm on mandatory 72-hour cyber incident reporting and 90-day forensic image preservation per DoD DFARS 252.204-7012(c) statutory flow-down (94% Held Firm precedent across 16 Tier-1 deals).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>EVT-8921-004</t>
+          <t>EVT-SP3-04-1792512543</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T22:37:23.971614+00:00</t>
+          <t>2026-10-20T16:09:03Z</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -3322,22 +3322,22 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>SP5-03</t>
+          <t>SP3-04</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>CYBER</t>
+          <t>TAX</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Capt. Devon Brooks (Lead, Supplier Cyber Defense)</t>
+          <t>Pradeep Gupta</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>SME_APPROVED</t>
+          <t>SME_POSITION_RECORDED</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -3347,19 +3347,19 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Enforced DFARS 252.204-7012 mandatory 72-hour cyber incident reporting lockout (94% held firm across 16 precedents).</t>
+          <t>Harmonized cross-clause conflict with GP1 §3.1 ($45M FFP ceiling): 50/50 shared tariff split above 5.0% threshold, strictly capped at +2.0% ($900,000) of the Firm-Fixed-Price SOW value (63% BigQuery precedent).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>EVT-8921-003</t>
+          <t>EVT-SP3-04-1792512541</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T22:32:23.971614+00:00</t>
+          <t>2026-10-20T16:09:01Z</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -3369,44 +3369,44 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>GP1-19</t>
+          <t>SP3-04</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>LEGAL</t>
+          <t>TAX</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Elena Rostova, J.D. (Senior Counsel, Commercial &amp; IP)</t>
+          <t>Pradeep Gupta</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>SME_APPROVED</t>
+          <t>SME_POSITION_RECORDED</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>compromise_tier_1</t>
+          <t>hold_firm</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>Selected Playbook Tier-1 Compromise (2x PO $90M super-cap + narrowed Cymbal Aerospace sole-spec IP carveout; 69% Tier-1 precedent).</t>
+          <t>Harmonized cross-clause conflict with GP1 §3.1 ($45M FFP ceiling): 50/50 shared tariff split above 5.0% threshold, strictly capped at +2.0% ($900,000) of the Firm-Fixed-Price SOW value (63% BigQuery precedent).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>EVT-8921-002</t>
+          <t>EVT-SP3-04-1792512539</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19T22:26:23.971614+00:00</t>
+          <t>2026-10-20T16:08:59Z</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3416,77 +3416,312 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>GP1-12</t>
+          <t>SP3-04</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>ENGINEERING</t>
+          <t>TAX</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Dr. Aris Thorne (Principal FAA DER, Flight Controls QA)</t>
+          <t>Pradeep Gupta</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>SME_APPROVED</t>
+          <t>SME_POSITION_RECORDED</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>hold_firm</t>
+          <t>compromise_tier_1</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Enforced FAA 14 CFR Part 21.140 unannounced inspection lockout and 36-month warranty (88% held firm across 16 precedents).</t>
+          <t>Harmonized cross-clause conflict with GP1 §3.1 ($45M FFP ceiling): 50/50 shared tariff split above 5.0% threshold, strictly capped at +2.0% ($900,000) of the Firm-Fixed-Price SOW value (63% BigQuery precedent).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
+          <t>EVT-GP1-12-1792509028</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-20T15:10:28Z</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>BA-2026-AV-8921</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>GP1-12</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>ENGINEERING</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Megan Bowen</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>SME_POSITION_RECORDED</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>hold_firm</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Rejected vendor 12-month warranty and 30-day inspection notice. FAA 14 CFR Part 21.140 and AS9100 Rev D mandate unannounced source inspection access at all times. Precedent shows 88% (14/16) held firm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>EVT-8921-005</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-19T22:43:23.971614+00:00</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>BA-2026-AV-8921</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>SP3-04</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>TAX</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Marcus Chen, CPA (Director, Global Tax &amp; Trade)</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>CONFLICT_TRIGGERED</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>accept_vendor</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Global Tax acceptance of uncapped &gt;5% Section 232/301 tariff pass-through triggered CRITICAL_CONFLICT with GP1 §3.1 Firm-Fixed-Price SOW Cap ($45M ceiling).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>EVT-8921-004</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-19T22:37:23.971614+00:00</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>BA-2026-AV-8921</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>SP5-03</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>CYBER</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Capt. Devon Brooks (Lead, Supplier Cyber Defense)</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>SME_APPROVED</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>hold_firm</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Enforced DFARS 252.204-7012 mandatory 72-hour cyber incident reporting lockout (94% held firm across 16 precedents).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>EVT-8921-003</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-19T22:32:23.971614+00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>BA-2026-AV-8921</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>GP1-19</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>LEGAL</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Elena Rostova, J.D. (Senior Counsel, Commercial &amp; IP)</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>SME_APPROVED</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>compromise_tier_1</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Selected Playbook Tier-1 Compromise (2x PO $90M super-cap + narrowed Cymbal Aerospace sole-spec IP carveout; 69% Tier-1 precedent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>EVT-8921-002</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-19T22:26:23.971614+00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>BA-2026-AV-8921</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>GP1-12</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>ENGINEERING</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Dr. Aris Thorne (Principal FAA DER, Flight Controls QA)</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>SME_APPROVED</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>hold_firm</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Enforced FAA 14 CFR Part 21.140 unannounced inspection lockout and 36-month warranty (88% held firm across 16 precedents).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>EVT-8921-001</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>2026-10-19T22:19:23.971614+00:00</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>BA-2026-AV-8921</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>PROCUREMENT</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Lead Contract Owner (M. Vance)</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>INGESTED_REDLINE</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>hold_firm</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>Deterministic OOXML Track Changes extraction completed against Cymbal_GP1_Standard.docx.</t>
         </is>

</xml_diff>